<commit_message>
factura-ia docs: rebrand Factu IA en TAREAS-PENDIENTES.xlsx
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sites/factura-ia/docs/TAREAS-PENDIENTES.xlsx
+++ b/sites/factura-ia/docs/TAREAS-PENDIENTES.xlsx
@@ -539,7 +539,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Landing de Factura IA — Estado del proyecto</t>
+          <t>Landing de Factu IA — Estado del proyecto</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>El logotipo de Factura IA se desalinea respecto a las columnas del pie.</t>
+          <t>El logotipo de Factu IA se desalinea respecto a las columnas del pie.</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>Falta el archivo assets/og-facturaia.jpg que referencia el og:image del index. Hoy, compartir el enlace por WhatsApp o Facebook no muestra imagen de vista previa.</t>
+          <t>Falta el archivo assets/og-factuia.jpg que referencia el og:image del index. Hoy, compartir el enlace por WhatsApp o Facebook no muestra imagen de vista previa.</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">

</xml_diff>